<commit_message>
Add README Benchmark & fix README print
</commit_message>
<xml_diff>
--- a/output_files/deliveries_analysis.xlsx
+++ b/output_files/deliveries_analysis.xlsx
@@ -7425,7 +7425,7 @@
         </is>
       </c>
       <c r="B1001" s="2">
-        <v>45870.48824074074</v>
+        <v>45884.54251157407</v>
       </c>
       <c r="C1001" t="inlineStr">
         <is>
@@ -7433,29 +7433,29 @@
         </is>
       </c>
       <c r="D1001">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E1001" t="inlineStr">
         <is>
-          <t>Special</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F1001">
-        <v>68.05</v>
+        <v>36.9</v>
       </c>
       <c r="G1001" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="H1001" t="inlineStr">
         <is>
-          <t>Snowy</t>
+          <t>Rainy</t>
         </is>
       </c>
       <c r="I1001" t="inlineStr">
         <is>
-          <t>138.18</t>
+          <t>105.42</t>
         </is>
       </c>
       <c r="J1001" t="inlineStr">

</xml_diff>